<commit_message>
refactor: update login route to redirect to sign-in and remove unused search button
</commit_message>
<xml_diff>
--- a/Connectly_Task_Tracker.xlsx
+++ b/Connectly_Task_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSLL4\OneDrive\Desktop\sachin\mern stack\Connectly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950038E7-1FEF-4BAC-935A-6DD847D73799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
   <si>
     <t>S.No</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>Contacts page build</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -517,8 +520,12 @@
       <c r="E2" s="4">
         <v>46317</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="F2" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G2" s="4">
+        <v>46317</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
@@ -588,13 +595,17 @@
         <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E6" s="4">
         <v>46317</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="F6" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G6" s="4">
+        <v>46317</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
@@ -612,8 +623,12 @@
       <c r="E7" s="4">
         <v>46317</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="F7" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G7" s="4">
+        <v>46317</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">

</xml_diff>

<commit_message>
fix: update text colors in ConversationPage and comment out group type display in ConversationsList
</commit_message>
<xml_diff>
--- a/Connectly_Task_Tracker.xlsx
+++ b/Connectly_Task_Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSLL4\OneDrive\Desktop\sachin\mern stack\Connectly\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aea0bc9152f7eeb2/Desktop/sachin/mern stack/Connectly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36EEA9DB-539C-4B51-82BF-C737A18ADABB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
     <t>Contacts page build</t>
   </si>
   <si>
-    <t>Done</t>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -95,7 +95,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,6 +113,12 @@
       <sz val="10"/>
       <color rgb="FF25324A"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF25324A"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -155,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -170,6 +176,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -617,8 +629,8 @@
       <c r="C7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
+      <c r="D7" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="E7" s="4">
         <v>46317</v>
@@ -668,7 +680,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -687,18 +699,18 @@
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+    <row r="11" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -870,7 +882,7 @@
   </sheetData>
   <autoFilter ref="A1:G9" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="C2:C200" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C10 C12:C200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Bug,Responsive,Feature Enhancement"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D2:D200" xr:uid="{00000000-0002-0000-0000-000001000000}">

</xml_diff>

<commit_message>
fix: update caret color for input fields and adjust timestamp display logic in ConversationPage
</commit_message>
<xml_diff>
--- a/Connectly_Task_Tracker.xlsx
+++ b/Connectly_Task_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aea0bc9152f7eeb2/Desktop/sachin/mern stack/Connectly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36EEA9DB-539C-4B51-82BF-C737A18ADABB}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6ADAF3C8-8D94-40B3-9E84-8D4D2266E57B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
   <si>
     <t>S.No</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>Completed</t>
+  </si>
+  <si>
+    <t>Not a Bug</t>
   </si>
 </sst>
 </file>
@@ -527,7 +530,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E2" s="4">
         <v>46317</v>

</xml_diff>

<commit_message>
schedule message bug fixed
</commit_message>
<xml_diff>
--- a/Connectly_Task_Tracker.xlsx
+++ b/Connectly_Task_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aea0bc9152f7eeb2/Desktop/sachin/mern stack/Connectly/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6ADAF3C8-8D94-40B3-9E84-8D4D2266E57B}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{70754793-0B19-4A7A-88E2-1178B70D16D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F5B8CC5-E9C9-4E2A-97C8-293ACDD30D39}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
   <si>
     <t>S.No</t>
   </si>
@@ -86,9 +86,6 @@
   </si>
   <si>
     <t>Completed</t>
-  </si>
-  <si>
-    <t>Not a Bug</t>
   </si>
 </sst>
 </file>
@@ -530,7 +527,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2" s="4">
         <v>46317</v>
@@ -553,13 +550,17 @@
         <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E3" s="4">
         <v>46317</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
+      <c r="F3" s="4">
+        <v>46319</v>
+      </c>
+      <c r="G3" s="4">
+        <v>46319</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">

</xml_diff>